<commit_message>
Export 4 new scripted videos + add export-status tracking to plan sheets
- SoftChic60: full scripts for "7 Boot Mistakes" and "6 Blouse Mistakes"
  (scripts-txt/02-boot-mistakes/, 03-blouse-mistakes/), appended to the
  content plan sheet.
- Viva Estilo: full scripts for "6 Relojes Elegantes" and "7 Formas de
  Usar un Pañuelo" (scripts-txt/02-relojes/, 03-panuelo/), appended to
  the content plan sheet.
- Both plan sheets gain a "Đã xuất content?" column marking which
  titles already have full scripts, so future research skips them.
- Update README with Viva Estilo entry; fill in Trendy & Timeless
  channel-info draft.
</commit_message>
<xml_diff>
--- a/channels/viva-estilo/output/vivaestilo-content-plan.xlsx
+++ b/channels/viva-estilo/output/vivaestilo-content-plan.xlsx
@@ -402,10 +402,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B32"/>
-  <cols>
-    <col min="1" max="1" width="42.83203125" customWidth="1"/>
-    <col min="2" max="2" width="95.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -658,18 +654,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J103"/>
-  <cols>
-    <col min="1" max="1" width="60.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="11.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="30.83203125" customWidth="1"/>
-    <col min="10" max="10" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3977,17 +3961,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I7"/>
-  <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="9.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="55.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4201,21 +4174,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
-  <cols>
-    <col min="1" max="1" width="4.83203125" customWidth="1"/>
-    <col min="2" max="2" width="9.83203125" customWidth="1"/>
-    <col min="3" max="3" width="55.83203125" customWidth="1"/>
-    <col min="4" max="4" width="35.83203125" customWidth="1"/>
-    <col min="5" max="5" width="45.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
-    <col min="8" max="8" width="45.83203125" customWidth="1"/>
-    <col min="9" max="9" width="55.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="35.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:M11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4254,6 +4213,9 @@
       <c r="L1" t="str">
         <v>Trạng thái</v>
       </c>
+      <c r="M1" t="str">
+        <v>Đã xuất content?</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -4292,6 +4254,9 @@
       <c r="L2" t="str">
         <v>Giai đoạn 1 — chờ duyệt trước khi viết kịch bản Giai đoạn 2 (tiếng TBN, theo template)</v>
       </c>
+      <c r="M2" t="str">
+        <v>✅ Đã xuất (kịch bản đầy đủ + ảnh)</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -4330,6 +4295,9 @@
       <c r="L3" t="str">
         <v>Giai đoạn 1 — chờ duyệt trước khi viết kịch bản Giai đoạn 2 (tiếng TBN, theo template)</v>
       </c>
+      <c r="M3" t="str">
+        <v>Chưa xuất</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -4368,6 +4336,9 @@
       <c r="L4" t="str">
         <v>Giai đoạn 1 — chờ duyệt trước khi viết kịch bản Giai đoạn 2 (tiếng TBN, theo template)</v>
       </c>
+      <c r="M4" t="str">
+        <v>Chưa xuất</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -4406,6 +4377,9 @@
       <c r="L5" t="str">
         <v>Giai đoạn 1 — chờ duyệt trước khi viết kịch bản Giai đoạn 2 (tiếng TBN, theo template)</v>
       </c>
+      <c r="M5" t="str">
+        <v>Chưa xuất</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -4444,6 +4418,9 @@
       <c r="L6" t="str">
         <v>Giai đoạn 1 — chờ duyệt trước khi viết kịch bản Giai đoạn 2 (tiếng TBN, theo template)</v>
       </c>
+      <c r="M6" t="str">
+        <v>Chưa xuất</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -4482,6 +4459,9 @@
       <c r="L7" t="str">
         <v>Giai đoạn 1 — chờ duyệt trước khi viết kịch bản Giai đoạn 2 (tiếng TBN, theo template)</v>
       </c>
+      <c r="M7" t="str">
+        <v>Chưa xuất</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -4520,6 +4500,9 @@
       <c r="L8" t="str">
         <v>Giai đoạn 1 — chờ duyệt trước khi viết kịch bản Giai đoạn 2 (tiếng TBN, theo template)</v>
       </c>
+      <c r="M8" t="str">
+        <v>Chưa xuất</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -4558,10 +4541,97 @@
       <c r="L9" t="str">
         <v>Giai đoạn 1 — chờ duyệt trước khi viết kịch bản Giai đoạn 2 (tiếng TBN, theo template)</v>
       </c>
+      <c r="M9" t="str">
+        <v>Chưa xuất</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Tuần 5</v>
+      </c>
+      <c r="C10" t="str">
+        <v>6 Relojes Elegantes que Te Hacen Ver RICA Después de los 60 (y 2 que Debes Evitar)</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Accesorio de muñeca — nunca cubierto en los 102 videos del canal ni en el plan actual; extiende el ángulo "verte rica" que ya funciona bien con bolsos y joyas.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>El formato "combo positivo + N que evitar" replica el patrón usado en los títulos de Zapatos y Joyas del propio plan (mismo canal), que siguen la fórmula de mayor rendimiento del nicho.</v>
+      </c>
+      <c r="F10" t="str">
+        <v>La piel de la muñeca cambia después de los 60 igual que la de las manos (se afina, se marcan venas) — un reloj bien elegido puede compensar ese cambio, tal como ya se demostró con el color de uñas.</v>
+      </c>
+      <c r="G10" t="str">
+        <v>El reloj como joya funcional: menos accesorios, más impacto.</v>
+      </c>
+      <c r="H10" t="str">
+        <v>6 relojes que favorecen la muñeca madura + 2 que conviene evitar.</v>
+      </c>
+      <c r="I10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hay un accesorio que muchas mujeres dejan en piloto automático, el mismo reloj de siempre, sin darse cuenta de que es una de las primeras cosas que alguien nota al saludarte con la mano, al servir el café o al gesticular mientras hablas: el reloj que llevas en la muñeca. Después de los sesenta, la piel de la muñeca cambia igual que la de las manos: se afina, se marcan más las venas, y un reloj que antes pasaba desapercibido de pronto puede jugar en tu contra o, todo lo contrario, favorecerte de una forma que ni imaginabas.
+No se trata de comprar el reloj más caro que encuentres, ni de tener seis relojes distintos para seis ocasiones. Se trata de algo mucho más simple: elegir la esfera, el tono y la correa correctos para que tu muñeca luzca elegante, cuidada y con esa seguridad que solo dan los años. Hoy quiero mostrarte seis relojes que de verdad te favorecen después de los sesenta, y antes de terminar, también te voy a contar cuáles son los dos que conviene dejar atrás, aunque los hayas usado toda la vida.</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Video largo, 12-15 min, formato lista con cierre de "evitar"</v>
+      </c>
+      <c r="K10" t="str">
+        <v>relojes elegantes mujeres 60, accesorios mujer madura, moda después de los 60, relojes que favorecen, estilo elegante 60 años</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Giai đoạn 2 hoàn tất — kịch bản đầy đủ + ảnh đã xuất theo yêu cầu trực tiếp của người dùng (bỏ qua bước chờ duyệt Giai đoạn 1 như thường lệ)</v>
+      </c>
+      <c r="M10" t="str">
+        <v>✅ Đã xuất (kịch bản đầy đủ + ảnh)</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Tuần 5</v>
+      </c>
+      <c r="C11" t="str">
+        <v>7 Formas de Usar un Pañuelo que Te Hacen Ver Elegante Después de los 50</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Accesorio de pañuelo/bufanda — nunca cubierto en los 102 videos del canal ni en el plan actual; aprovecha un accesorio infrautilizado pero de bajo costo de producción.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Belleza Serena (207K sub) es fuerte en accesorios/tocados; formato de "lista de usos" del mismo accesorio no ha sido probado en Viva Estilo todavía.</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Muchas mujeres tienen pañuelos de seda guardados sin usar porque no saben cómo llevarlos — el video resuelve un "no sé cómo" muy concreto y accionable.</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Un mismo pañuelo, siete formas distintas — versatilidad y bajo costo.</v>
+      </c>
+      <c r="H11" t="str">
+        <v>7 formas de anudar/usar un pañuelo para verte elegante después de los 50.</v>
+      </c>
+      <c r="I11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hay un accesorio que muchas mujeres tienen guardado en un cajón, heredado de su madre o comprado por impulso en un viaje, y que casi nunca se atreven a usar porque no saben bien cómo: el pañuelo. Después de los cincuenta, ese mismo pañuelo que parece "demasiado sofisticado" para el día a día puede convertirse justo en el detalle que transforma un look sencillo en uno con clase, sin gastar un euro más.
+No se trata de convertirte en una experta en nudos franceses complicados, ni de comprar diez pañuelos distintos. Se trata de siete formas simples de llevarlo que puedes aprender hoy mismo, cada una en menos de un minuto, usando el pañuelo que probablemente ya tienes guardado en algún cajón.</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Video largo, 10-13 min, formato lista con demostración práctica por forma</v>
+      </c>
+      <c r="K11" t="str">
+        <v>como usar un pañuelo, accesorios mujer después de los 50, moda elegante 50 años, pañuelo de seda outfit, estilo atemporal</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Giai đoạn 2 hoàn tất — kịch bản đầy đủ + ảnh đã xuất theo yêu cầu trực tiếp của người dùng (bỏ qua bước chờ duyệt Giai đoạn 1 như thường lệ)</v>
+      </c>
+      <c r="M11" t="str">
+        <v>✅ Đã xuất (kịch bản đầy đủ + ảnh)</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4569,12 +4639,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D6"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="70.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>